<commit_message>
feat: vista real acumulado unificada, HH/ing/gasto real por línea y acceso por módulo
- Fusiona VistaIngresoRealAcumulado y VistaGastoRealAcumulado en VistaRealAcumulado (una sola carga con columnas Proyecto, Ingreso y Gasto)
- Modal de confirmación muestra solo proyectos sin match en tabla de proyectos
- Seguimiento Operacional: HH, Ingreso y Gasto real vienen de Supabase agrupados por línea
- Control de acceso por módulo: columna modulos TEXT[] en perfiles, canSee() en App.jsx
- Migración 20260611120000: agrega columna modulos a perfiles

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/ppto2026.xlsx
+++ b/public/ppto2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fchnew-my.sharepoint.com/personal/emilio_lopez_fch_cl/Documents/Documentos/Proyectos/gestion-proyectos-fch/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fchnew-my.sharepoint.com/personal/emilio_lopez_fch_cl/Documents/Documentos/Proyectos/gestion-proyectos-fch/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="8_{C7F785CD-F492-45A6-8011-A052CA213773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FDE25C3-2083-4319-BD31-89B6ED5F458D}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="8_{C7F785CD-F492-45A6-8011-A052CA213773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD1363C8-B81B-4A52-B5EF-14FBB25CE35D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{455D1B75-5C12-4E50-9089-0B0A661360FD}"/>
   </bookViews>
@@ -700,12 +700,11 @@
   <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.6328125" customWidth="1"/>
     <col min="2" max="2" width="43.08984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.08984375" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="13.26953125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.90625" bestFit="1" customWidth="1"/>
   </cols>
@@ -1737,7 +1736,7 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>45</v>
@@ -1768,7 +1767,7 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>46</v>
@@ -1797,7 +1796,7 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>47</v>
@@ -1826,7 +1825,7 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>48</v>
@@ -1859,7 +1858,7 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>49</v>
@@ -1888,7 +1887,7 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>50</v>
@@ -1917,7 +1916,7 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>51</v>
@@ -1946,7 +1945,7 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>52</v>
@@ -1975,7 +1974,7 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>53</v>
@@ -2004,7 +2003,7 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>54</v>
@@ -2033,7 +2032,7 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>55</v>
@@ -2064,7 +2063,7 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>56</v>

</xml_diff>